<commit_message>
Added patch to sync codebase with deployed application tweaks.
</commit_message>
<xml_diff>
--- a/backend/Dataset/customers.xlsx
+++ b/backend/Dataset/customers.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/whm208_exeter_ac_uk/Documents/Year 2/COM2020/Coursework 1/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="8_{7A4EF343-2723-4A7C-9B60-C82987C01CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7BB608D-78D8-40A2-9AD1-286649AA9523}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="8_{7A4EF343-2723-4A7C-9B60-C82987C01CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{098C7EC7-DA26-415B-95CC-AE16A9BE429C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{419C08BF-9424-4E75-98EB-76D780432850}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>customerID</t>
   </si>
@@ -132,18 +132,12 @@
   </si>
   <si>
     <t>customer60</t>
-  </si>
-  <si>
-    <t>creationDate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
-  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -196,11 +190,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -539,352 +532,258 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F61BE75-A0CC-4778-AF2F-846F6990A8A0}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>32</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>34</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>37</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>38</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>39</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>40</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>41</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>42</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>43</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>46</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>47</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>48</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>49</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>50</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>51</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>52</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>53</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>54</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>55</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>56</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>57</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>58</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>59</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="3">
-        <v>45292</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>60</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="C31" s="3">
-        <v>45292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>